<commit_message>
Add Activity_Type column to Master_Inputs (Baseline | Strategy)
New column at position H (between Source_Document and Provenance).
Default = Baseline. Dropdown values: Baseline | Strategy.

Captures the row classification orthogonally from Source_Document:
- Baseline = ongoing recurring activity (W-2, K-1, dividends, etc.)
- Strategy = committed tax planning move (Cost Seg, Augusta, etc.)

Sample data updated:
- All existing rows tagged Activity_Type = "Baseline"
- New sample row added (SAM|2025|Strategy|CostSeg|01) showing a
  committed Cost Seg study with Activity_Type = "Strategy",
  Treatment_Profile = "SchE_Rental", Baseline_Amount = -80000,
  flowing through Bucket = Business Income → Primary_Line = 8.

Pivots are unchanged — they'll include all rows by default. Future:
add SUMIFS filter clause "...tblMaster_Inputs[Activity_Type], 'Baseline'"
when you want the baseline-only view. Workbook-level named range
Activity_Type points at the dropdown list for data validation.
</commit_message>
<xml_diff>
--- a/docs/Master_Pivot_Framework.xlsx
+++ b/docs/Master_Pivot_Framework.xlsx
@@ -23,6 +23,7 @@
     <definedName name="Provenance">'Dropdown_Lists'!$D$4:$D$13</definedName>
     <definedName name="Status">'Dropdown_Lists'!$E$4:$E$8</definedName>
     <definedName name="TaxLines">'Dropdown_Lists'!$F$4:$F$13</definedName>
+    <definedName name="Activity_Type">'Dropdown_Lists'!$G$4:$G$5</definedName>
     <definedName name="BusinessIncome_Profiles">'Dropdown_Lists'!$A$19:$A$27</definedName>
     <definedName name="Wages_Profiles">'Dropdown_Lists'!$B$19:$B$20</definedName>
     <definedName name="InvestmentIncome_Profiles">'Dropdown_Lists'!$C$19:$C$22</definedName>
@@ -262,9 +263,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblMaster_Inputs" displayName="tblMaster_Inputs" ref="A4:R14" headerRowCount="1">
-  <autoFilter ref="A4:R14"/>
-  <tableColumns count="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblMaster_Inputs" displayName="tblMaster_Inputs" ref="A4:S15" headerRowCount="1">
+  <autoFilter ref="A4:S15"/>
+  <tableColumns count="19">
     <tableColumn id="1" name="InputID"/>
     <tableColumn id="2" name="Year"/>
     <tableColumn id="3" name="ClientID"/>
@@ -272,17 +273,18 @@
     <tableColumn id="5" name="Bucket"/>
     <tableColumn id="6" name="Treatment_Profile"/>
     <tableColumn id="7" name="Source_Document"/>
-    <tableColumn id="8" name="Provenance"/>
-    <tableColumn id="9" name="Payor"/>
-    <tableColumn id="10" name="Baseline_Amount"/>
-    <tableColumn id="11" name="Helper_Amount"/>
-    <tableColumn id="12" name="SE_Subject"/>
-    <tableColumn id="13" name="NIIT_Class"/>
-    <tableColumn id="14" name="QBI_Eligible"/>
-    <tableColumn id="15" name="Primary_Line"/>
-    <tableColumn id="16" name="Helper_Treatment"/>
-    <tableColumn id="17" name="Consider"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="8" name="Activity_Type"/>
+    <tableColumn id="9" name="Provenance"/>
+    <tableColumn id="10" name="Payor"/>
+    <tableColumn id="11" name="Baseline_Amount"/>
+    <tableColumn id="12" name="Helper_Amount"/>
+    <tableColumn id="13" name="SE_Subject"/>
+    <tableColumn id="14" name="NIIT_Class"/>
+    <tableColumn id="15" name="QBI_Eligible"/>
+    <tableColumn id="16" name="Primary_Line"/>
+    <tableColumn id="17" name="Helper_Treatment"/>
+    <tableColumn id="18" name="Consider"/>
+    <tableColumn id="19" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -610,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -620,17 +622,18 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -685,55 +688,60 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>Activity_Type</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Provenance</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Payor</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Baseline_Amount</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Helper_Amount</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>SE_Subject</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>NIIT_Class</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>QBI_Eligible</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Primary_Line</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Helper_Treatment</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Consider</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -775,51 +783,56 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
           <t>PBC - Reviewed</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Acme S-Corp</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>153648</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
           <t>1z</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>OWNER_PAY</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t>Owner reasonable comp</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -857,51 +870,56 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
           <t>PBC - Reviewed</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Cedillo Partnership</t>
         </is>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>-100766</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
           <t>Passive</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>K1_SPLIT</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>Passive loss</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -939,51 +957,56 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
           <t>PBC - Reviewed</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Brokerage</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>25922</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
           <t>3b</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>QUAL_DIV</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>All non-qualified</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1021,51 +1044,56 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
           <t>PBC - Reviewed</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Brokerage</t>
         </is>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>14487</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>LTCG_SPLIT</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t>All long-term</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1103,51 +1131,56 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
           <t>Estimate - Preparer</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>SampleCo S-Corp</t>
         </is>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>100000</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>100000</v>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+      <c r="L9" s="4" t="n">
+        <v>100000</v>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
           <t>1z</t>
         </is>
       </c>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>OWNER_PAY</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>Owner reasonable comp</t>
         </is>
       </c>
-      <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1185,51 +1218,56 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
           <t>PY Rolled Forward</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>SampleCo S-Corp K-1</t>
         </is>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>200000</v>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="L10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>K1_SPLIT</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>Active S-corp K-1</t>
         </is>
       </c>
-      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1267,51 +1305,56 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
           <t>PBC - Received</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Brokerage</t>
         </is>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>7000</v>
       </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
           <t>3b</t>
         </is>
       </c>
-      <c r="P11" s="4" t="inlineStr">
+      <c r="Q11" s="4" t="inlineStr">
         <is>
           <t>QUAL_DIV</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="inlineStr">
+      <c r="R11" s="4" t="inlineStr">
         <is>
           <t>$7K qualified</t>
         </is>
       </c>
-      <c r="R11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1349,51 +1392,56 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
           <t>PBC - Received</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Brokerage</t>
         </is>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>500</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
           <t>2b</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>TAX_EXEMPT</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="R12" s="4" t="inlineStr">
         <is>
           <t>All taxable</t>
         </is>
       </c>
-      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1431,51 +1479,56 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
           <t>PBC - Requested</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Brokerage</t>
         </is>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="K13" s="4" t="n">
         <v>25000</v>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="L13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>LTCG_SPLIT</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="R13" s="4" t="inlineStr">
         <is>
           <t>All long-term</t>
         </is>
       </c>
-      <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1513,50 +1566,138 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
           <t>PBC - Received</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="n">
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>SALT</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr">
         <is>
           <t>SALT cap</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>SAM|2025|Strategy|CostSeg|01</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>SAMPLE</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Sample Client</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Business Income</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>SchE_Rental</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Estimate - Preparer</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="n">
+        <v>-80000</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>PASSIVE</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>Cost Seg accelerated depreciation</t>
+        </is>
+      </c>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>STD-012 Committed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation sqref="E5:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Bucket</formula1>
     </dataValidation>
@@ -1567,15 +1708,18 @@
       <formula1>=INDIRECT(SUBSTITUTE($E5," ","")&amp;"_Docs")</formula1>
     </dataValidation>
     <dataValidation sqref="H5:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Activity_Type</formula1>
+    </dataValidation>
+    <dataValidation sqref="I5:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Provenance</formula1>
     </dataValidation>
-    <dataValidation sqref="L5:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M5:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Yes_No</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N5:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=NIIT_Class</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O5:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Yes_No</formula1>
     </dataValidation>
   </dataValidations>
@@ -6737,6 +6881,11 @@
           <t>TaxLines</t>
         </is>
       </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Activity_Type</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6769,6 +6918,11 @@
           <t>1z</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6799,6 +6953,11 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>2a</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Strategy</t>
         </is>
       </c>
     </row>

</xml_diff>